<commit_message>
Finalize AIIO public prototype gate
</commit_message>
<xml_diff>
--- a/public/downloads/AIIO_Alberta_Pilot_0.2.0-dev.xlsx
+++ b/public/downloads/AIIO_Alberta_Pilot_0.2.0-dev.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="1" r:id="Rb838b13b0bac407c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="Rc7dd6c4ba830483e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="3" r:id="R9980c1a238104b31"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenario Timeline" sheetId="4" r:id="R2e3058dbcbf14548"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pressure Results" sheetId="5" r:id="Rc32b87ea3fe84589"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="6" r:id="R489d4e8b19774908"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Power Overlay" sheetId="7" r:id="R1d2cc36515e64099"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI Projects" sheetId="8" r:id="R1310427029d14b0e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BCPI Data" sheetId="9" r:id="Rdc723795255a46d7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="10" r:id="R672db09ac6e64b79"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Checks" sheetId="11" r:id="Rf51c4ea08a824eef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="1" r:id="Rbdb659b915764819"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="R2e69be1753184ee9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="3" r:id="R48d9bf2bb64540ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenario Timeline" sheetId="4" r:id="R878b963625d4435b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pressure Results" sheetId="5" r:id="Raad432c252a24166"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="6" r:id="R82df74d975344d32"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Power Overlay" sheetId="7" r:id="Rc5cf58c9d7284230"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI Projects" sheetId="8" r:id="Rda3802c712c44f98"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BCPI Data" sheetId="9" r:id="R15f4ea50a4544859"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="10" r:id="R3aaf5d4183144220"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Checks" sheetId="11" r:id="Rd3445bf53d9a4991"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -20,9 +20,9 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:comments xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:authors>
-    <x:author>tc={798204B1-73D1-4CC6-A3A2-58A5552F13C2}</x:author>
-    <x:author>tc={9B3FE770-F6B8-4F6F-9886-CB2ADF8F8FC8}</x:author>
-    <x:author>tc={D9469942-DA12-4E7E-9712-C91FE571C553}</x:author>
+    <x:author>tc={885C3C5E-B985-4690-9C8E-99BA6A8408ED}</x:author>
+    <x:author>tc={D0D9660F-855D-4070-8175-EF5C94D0680C}</x:author>
+    <x:author>tc={BDA8B6C9-D04B-47AC-864D-F116A333B949}</x:author>
   </x:authors>
   <x:commentList>
     <x:comment ref="B5" authorId="0">
@@ -1360,7 +1360,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rd1d97b7d993745b1"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R59d3b6fddc964358"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1390,7 +1390,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Ra2d6c480c1d34197"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R9706369f0cd44566"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1418,7 +1418,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:personList xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:person displayName="User" id="{F8493558-F1F6-41C7-A408-3AE737B83E7A}"/>
+  <xltc:person displayName="User" id="{598A9BB0-9441-48FB-A7E6-D669CE17B875}"/>
 </xltc:personList>
 </file>
 
@@ -1691,13 +1691,13 @@
 
 <file path=xl/threadedcomments/threadedcomment.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:ThreadedComments xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:threadedComment ref="B5" dT="2026-08-31T15:06:57.405" personId="{F8493558-F1F6-41C7-A408-3AE737B83E7A}" id="{798204B1-73D1-4CC6-A3A2-58A5552F13C2}">
+  <xltc:threadedComment ref="B5" dT="2026-08-31T15:29:59.987" personId="{598A9BB0-9441-48FB-A7E6-D669CE17B875}" id="{885C3C5E-B985-4690-9C8E-99BA6A8408ED}">
     <xltc:text>Scenario-only input. This is not a forecast or a total of committed projects.</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="B10" dT="2026-08-31T15:06:57.405" personId="{F8493558-F1F6-41C7-A408-3AE737B83E7A}" id="{9B3FE770-F6B8-4F6F-9886-CB2ADF8F8FC8}">
+  <xltc:threadedComment ref="B10" dT="2026-08-31T15:29:59.988" personId="{598A9BB0-9441-48FB-A7E6-D669CE17B875}" id="{D0D9660F-855D-4070-8175-EF5C94D0680C}">
     <xltc:text>Assumed share of locally captured construction and service demand. Test through sensitivity analysis before interpretation.</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="C24" dT="2026-08-31T15:06:57.405" personId="{F8493558-F1F6-41C7-A408-3AE737B83E7A}" id="{D9469942-DA12-4E7E-9712-C91FE571C553}">
+  <xltc:threadedComment ref="C24" dT="2026-08-31T15:29:59.988" personId="{598A9BB0-9441-48FB-A7E6-D669CE17B875}" id="{BDA8B6C9-D04B-47AC-864D-F116A333B949}">
     <xltc:text>IT load is an independent power-case assumption. It is not derived from capital expenditure.</xltc:text>
   </xltc:threadedComment>
 </xltc:ThreadedComments>
@@ -2540,7 +2540,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd98578f4d0dd4ac4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc2bd8cb1597e4c71"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2648,7 +2648,7 @@
         <x:v>Code commit</x:v>
       </x:c>
       <x:c r="B11" s="160" t="str">
-        <x:v>5bf68c25641cf3c8d2291760d1975486f4e31323</x:v>
+        <x:v>9812157428b38e578291a31e1a4eb43b6e9d8ec7</x:v>
       </x:c>
       <x:c r="C11" s="63"/>
       <x:c r="D11" s="63"/>
@@ -2658,7 +2658,7 @@
         <x:v>Input manifest hash</x:v>
       </x:c>
       <x:c r="B12" s="160" t="str">
-        <x:v>sha256:78d80249d4748d8f5f2586b90ddea3456ea7433c49dab3fbdd1d271c57cc55f5</x:v>
+        <x:v>sha256:88911fcc418a171c66bbe1ad100835dbfc28f4975798a1489e4ee758e4c53c09</x:v>
       </x:c>
       <x:c r="C12" s="63"/>
       <x:c r="D12" s="63"/>
@@ -2937,7 +2937,7 @@
       <x:c r="F6" s="232"/>
       <x:c r="G6" s="234" t="n">
         <x:f>MAX('Pressure Results'!$F$5:$F$8)</x:f>
-        <x:v>0.62</x:v>
+        <x:v>0.3827</x:v>
       </x:c>
       <x:c r="H6" s="231"/>
       <x:c r="I6" s="232"/>
@@ -3001,7 +3001,7 @@
       </x:c>
       <x:c r="B10" s="147" t="n">
         <x:f>'Pressure Results'!F5</x:f>
-        <x:v>0.62</x:v>
+        <x:v>0.3827</x:v>
       </x:c>
       <x:c r="C10" s="63"/>
       <x:c r="D10" s="63"/>
@@ -3021,7 +3021,7 @@
       </x:c>
       <x:c r="B11" s="147" t="n">
         <x:f>'Pressure Results'!F6</x:f>
-        <x:v>0.42</x:v>
+        <x:v>0.2958</x:v>
       </x:c>
       <x:c r="C11" s="63"/>
       <x:c r="D11" s="63"/>
@@ -3041,7 +3041,7 @@
       </x:c>
       <x:c r="B12" s="147" t="n">
         <x:f>'Pressure Results'!F7</x:f>
-        <x:v>0.29</x:v>
+        <x:v>0.2248</x:v>
       </x:c>
       <x:c r="C12" s="63"/>
       <x:c r="D12" s="63"/>
@@ -3061,7 +3061,7 @@
       </x:c>
       <x:c r="B13" s="147" t="n">
         <x:f>'Pressure Results'!F8</x:f>
-        <x:v>0.25</x:v>
+        <x:v>0.2</x:v>
       </x:c>
       <x:c r="C13" s="63"/>
       <x:c r="D13" s="63"/>
@@ -3562,7 +3562,7 @@
     </x:row>
     <x:row r="44">
       <x:c r="A44" s="240" t="str">
-        <x:v>Release hash: sha256:78d80249d4748d8f5f2586b90ddea3456ea7433c49dab3fbdd1d271c57cc55f5</x:v>
+        <x:v>Release hash: sha256:88911fcc418a171c66bbe1ad100835dbfc28f4975798a1489e4ee758e4c53c09</x:v>
       </x:c>
       <x:c r="B44" s="63"/>
       <x:c r="C44" s="63"/>
@@ -3592,7 +3592,7 @@
     <x:mergeCell ref="A44:L44"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6cbe9cb872b84570"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf55b22b0dcb0489d"/>
 </x:worksheet>
 </file>
 
@@ -4329,7 +4329,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rffc2daf7e89f49a1"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf0b9b4e894ad4702"/>
 </x:worksheet>
 </file>
 
@@ -4901,19 +4901,19 @@
         <x:v>resource</x:v>
       </x:c>
       <x:c r="D5" s="147" t="n">
-        <x:v>0.33</x:v>
+        <x:v>0.2481</x:v>
       </x:c>
       <x:c r="E5" s="63" t="n">
         <x:v>2033</x:v>
       </x:c>
       <x:c r="F5" s="147" t="n">
-        <x:v>0.62</x:v>
+        <x:v>0.3827</x:v>
       </x:c>
       <x:c r="G5" s="63" t="n">
         <x:v>2034</x:v>
       </x:c>
       <x:c r="H5" s="147" t="n">
-        <x:v>1.23</x:v>
+        <x:v>0.5516</x:v>
       </x:c>
       <x:c r="I5" s="63" t="n">
         <x:v>2035</x:v>
@@ -4939,19 +4939,19 @@
         <x:v>resource</x:v>
       </x:c>
       <x:c r="D6" s="147" t="n">
-        <x:v>0.2</x:v>
+        <x:v>0.1667</x:v>
       </x:c>
       <x:c r="E6" s="63" t="n">
         <x:v>2033</x:v>
       </x:c>
       <x:c r="F6" s="147" t="n">
-        <x:v>0.42</x:v>
+        <x:v>0.2958</x:v>
       </x:c>
       <x:c r="G6" s="63" t="n">
         <x:v>2034</x:v>
       </x:c>
       <x:c r="H6" s="147" t="n">
-        <x:v>0.89</x:v>
+        <x:v>0.4709</x:v>
       </x:c>
       <x:c r="I6" s="63" t="n">
         <x:v>2035</x:v>
@@ -4977,19 +4977,19 @@
         <x:v>resource</x:v>
       </x:c>
       <x:c r="D7" s="147" t="n">
-        <x:v>0.14</x:v>
+        <x:v>0.1228</x:v>
       </x:c>
       <x:c r="E7" s="63" t="n">
         <x:v>2033</x:v>
       </x:c>
       <x:c r="F7" s="147" t="n">
-        <x:v>0.29</x:v>
+        <x:v>0.2248</x:v>
       </x:c>
       <x:c r="G7" s="63" t="n">
         <x:v>2034</x:v>
       </x:c>
       <x:c r="H7" s="147" t="n">
-        <x:v>0.59</x:v>
+        <x:v>0.3711</x:v>
       </x:c>
       <x:c r="I7" s="63" t="n">
         <x:v>2035</x:v>
@@ -5015,19 +5015,19 @@
         <x:v>resource</x:v>
       </x:c>
       <x:c r="D8" s="147" t="n">
-        <x:v>0.12</x:v>
+        <x:v>0.1071</x:v>
       </x:c>
       <x:c r="E8" s="63" t="n">
         <x:v>2033</x:v>
       </x:c>
       <x:c r="F8" s="147" t="n">
-        <x:v>0.25</x:v>
+        <x:v>0.2</x:v>
       </x:c>
       <x:c r="G8" s="63" t="n">
         <x:v>2034</x:v>
       </x:c>
       <x:c r="H8" s="147" t="n">
-        <x:v>0.52</x:v>
+        <x:v>0.3421</x:v>
       </x:c>
       <x:c r="I8" s="63" t="n">
         <x:v>2035</x:v>
@@ -5053,19 +5053,19 @@
         <x:v>outcome</x:v>
       </x:c>
       <x:c r="D9" s="147" t="n">
-        <x:v>0.09</x:v>
+        <x:v>0.0826</x:v>
       </x:c>
       <x:c r="E9" s="63" t="n">
         <x:v>2034</x:v>
       </x:c>
       <x:c r="F9" s="147" t="n">
-        <x:v>0.45</x:v>
+        <x:v>0.3056</x:v>
       </x:c>
       <x:c r="G9" s="63" t="n">
         <x:v>2035</x:v>
       </x:c>
       <x:c r="H9" s="147" t="n">
-        <x:v>2.49</x:v>
+        <x:v>0.7041</x:v>
       </x:c>
       <x:c r="I9" s="63" t="n">
         <x:v>2038</x:v>
@@ -5091,19 +5091,19 @@
         <x:v>outcome</x:v>
       </x:c>
       <x:c r="D10" s="147" t="n">
-        <x:v>0.08</x:v>
+        <x:v>0.0654</x:v>
       </x:c>
       <x:c r="E10" s="63" t="n">
         <x:v>2034</x:v>
       </x:c>
       <x:c r="F10" s="147" t="n">
-        <x:v>0.36</x:v>
+        <x:v>0.2308</x:v>
       </x:c>
       <x:c r="G10" s="63" t="n">
         <x:v>2035</x:v>
       </x:c>
       <x:c r="H10" s="147" t="n">
-        <x:v>1.51</x:v>
+        <x:v>0.5536</x:v>
       </x:c>
       <x:c r="I10" s="63" t="n">
         <x:v>2037</x:v>
@@ -5129,19 +5129,19 @@
         <x:v>outcome</x:v>
       </x:c>
       <x:c r="D11" s="147" t="n">
-        <x:v>0.06</x:v>
+        <x:v>0.0476</x:v>
       </x:c>
       <x:c r="E11" s="63" t="n">
         <x:v>2034</x:v>
       </x:c>
       <x:c r="F11" s="147" t="n">
-        <x:v>0.29</x:v>
+        <x:v>0.2248</x:v>
       </x:c>
       <x:c r="G11" s="63" t="n">
         <x:v>2035</x:v>
       </x:c>
       <x:c r="H11" s="147" t="n">
-        <x:v>1.69</x:v>
+        <x:v>0.6169</x:v>
       </x:c>
       <x:c r="I11" s="63" t="n">
         <x:v>2038</x:v>
@@ -5167,19 +5167,19 @@
         <x:v>outcome</x:v>
       </x:c>
       <x:c r="D12" s="147" t="n">
-        <x:v>0.04</x:v>
+        <x:v>0.0385</x:v>
       </x:c>
       <x:c r="E12" s="63" t="n">
         <x:v>2034</x:v>
       </x:c>
       <x:c r="F12" s="147" t="n">
-        <x:v>0.23</x:v>
+        <x:v>0.1803</x:v>
       </x:c>
       <x:c r="G12" s="63" t="n">
         <x:v>2035</x:v>
       </x:c>
       <x:c r="H12" s="147" t="n">
-        <x:v>1.31</x:v>
+        <x:v>0.5556</x:v>
       </x:c>
       <x:c r="I12" s="63" t="n">
         <x:v>2038</x:v>
@@ -5205,19 +5205,19 @@
         <x:v>outcome</x:v>
       </x:c>
       <x:c r="D13" s="147" t="n">
-        <x:v>0.02</x:v>
+        <x:v>0.0196</x:v>
       </x:c>
       <x:c r="E13" s="63" t="n">
         <x:v>2034</x:v>
       </x:c>
       <x:c r="F13" s="147" t="n">
-        <x:v>0.12</x:v>
+        <x:v>0.1071</x:v>
       </x:c>
       <x:c r="G13" s="63" t="n">
         <x:v>2035</x:v>
       </x:c>
       <x:c r="H13" s="147" t="n">
-        <x:v>0.57</x:v>
+        <x:v>0.3631</x:v>
       </x:c>
       <x:c r="I13" s="63" t="n">
         <x:v>2037</x:v>
@@ -5504,7 +5504,7 @@
         <x:v>Building electricians</x:v>
       </x:c>
       <x:c r="I5" s="147" t="n">
-        <x:v>0.62</x:v>
+        <x:v>0.3827</x:v>
       </x:c>
       <x:c r="J5" s="63" t="n">
         <x:v>2034</x:v>
@@ -5513,7 +5513,7 @@
         <x:v>Hospital delivery delay pressure</x:v>
       </x:c>
       <x:c r="L5" s="147" t="n">
-        <x:v>0.45</x:v>
+        <x:v>0.3056</x:v>
       </x:c>
       <x:c r="M5" s="63" t="n">
         <x:v>2035</x:v>
@@ -5545,7 +5545,7 @@
         <x:v>Building electricians</x:v>
       </x:c>
       <x:c r="I6" s="147" t="n">
-        <x:v>1.23</x:v>
+        <x:v>0.5516</x:v>
       </x:c>
       <x:c r="J6" s="63" t="n">
         <x:v>2034</x:v>
@@ -5554,7 +5554,7 @@
         <x:v>Hospital delivery delay pressure</x:v>
       </x:c>
       <x:c r="L6" s="147" t="n">
-        <x:v>0.9</x:v>
+        <x:v>0.4681</x:v>
       </x:c>
       <x:c r="M6" s="63" t="n">
         <x:v>2035</x:v>
@@ -5586,7 +5586,7 @@
         <x:v>Building electricians</x:v>
       </x:c>
       <x:c r="I7" s="147" t="n">
-        <x:v>0.31</x:v>
+        <x:v>0.2366</x:v>
       </x:c>
       <x:c r="J7" s="63" t="n">
         <x:v>2034</x:v>
@@ -5595,7 +5595,7 @@
         <x:v>Hospital delivery delay pressure</x:v>
       </x:c>
       <x:c r="L7" s="147" t="n">
-        <x:v>0.22</x:v>
+        <x:v>0.1803</x:v>
       </x:c>
       <x:c r="M7" s="63" t="n">
         <x:v>2035</x:v>
@@ -5627,7 +5627,7 @@
         <x:v>Building electricians</x:v>
       </x:c>
       <x:c r="I8" s="147" t="n">
-        <x:v>0.69</x:v>
+        <x:v>0.4083</x:v>
       </x:c>
       <x:c r="J8" s="63" t="n">
         <x:v>2034</x:v>
@@ -5636,7 +5636,7 @@
         <x:v>Hospital delivery delay pressure</x:v>
       </x:c>
       <x:c r="L8" s="147" t="n">
-        <x:v>0.57</x:v>
+        <x:v>0.359</x:v>
       </x:c>
       <x:c r="M8" s="63" t="n">
         <x:v>2035</x:v>
@@ -5668,7 +5668,7 @@
         <x:v>Building electricians</x:v>
       </x:c>
       <x:c r="I9" s="147" t="n">
-        <x:v>0.55</x:v>
+        <x:v>0.3548</x:v>
       </x:c>
       <x:c r="J9" s="63" t="n">
         <x:v>2034</x:v>
@@ -5677,7 +5677,7 @@
         <x:v>Hospital delivery delay pressure</x:v>
       </x:c>
       <x:c r="L9" s="147" t="n">
-        <x:v>0.34</x:v>
+        <x:v>0.2537</x:v>
       </x:c>
       <x:c r="M9" s="63" t="n">
         <x:v>2035</x:v>
@@ -5709,7 +5709,7 @@
         <x:v>Building electricians</x:v>
       </x:c>
       <x:c r="I10" s="147" t="n">
-        <x:v>0.34</x:v>
+        <x:v>0.2537</x:v>
       </x:c>
       <x:c r="J10" s="63" t="n">
         <x:v>2034</x:v>
@@ -5718,7 +5718,7 @@
         <x:v>Hospital delivery delay pressure</x:v>
       </x:c>
       <x:c r="L10" s="147" t="n">
-        <x:v>0.25</x:v>
+        <x:v>0.1935</x:v>
       </x:c>
       <x:c r="M10" s="63" t="n">
         <x:v>2035</x:v>
@@ -5750,7 +5750,7 @@
         <x:v>Building electricians</x:v>
       </x:c>
       <x:c r="I11" s="147" t="n">
-        <x:v>0.77</x:v>
+        <x:v>0.435</x:v>
       </x:c>
       <x:c r="J11" s="63" t="n">
         <x:v>2034</x:v>
@@ -5759,7 +5759,7 @@
         <x:v>Hospital delivery delay pressure</x:v>
       </x:c>
       <x:c r="L11" s="147" t="n">
-        <x:v>0.56</x:v>
+        <x:v>0.3548</x:v>
       </x:c>
       <x:c r="M11" s="63" t="n">
         <x:v>2035</x:v>
@@ -5791,7 +5791,7 @@
         <x:v>Building electricians</x:v>
       </x:c>
       <x:c r="I12" s="147" t="n">
-        <x:v>0.41</x:v>
+        <x:v>0.2908</x:v>
       </x:c>
       <x:c r="J12" s="63" t="n">
         <x:v>2033</x:v>
@@ -5800,7 +5800,7 @@
         <x:v>Hospital delivery delay pressure</x:v>
       </x:c>
       <x:c r="L12" s="147" t="n">
-        <x:v>0.21</x:v>
+        <x:v>0.1736</x:v>
       </x:c>
       <x:c r="M12" s="63" t="n">
         <x:v>2034</x:v>
@@ -5832,7 +5832,7 @@
         <x:v>Building electricians</x:v>
       </x:c>
       <x:c r="I13" s="147" t="n">
-        <x:v>1.01</x:v>
+        <x:v>0.5025</x:v>
       </x:c>
       <x:c r="J13" s="63" t="n">
         <x:v>2035</x:v>
@@ -5841,7 +5841,7 @@
         <x:v>Hospital delivery delay pressure</x:v>
       </x:c>
       <x:c r="L13" s="147" t="n">
-        <x:v>1.24</x:v>
+        <x:v>0.5455</x:v>
       </x:c>
       <x:c r="M13" s="63" t="n">
         <x:v>2038</x:v>
@@ -5873,7 +5873,7 @@
         <x:v>Building electricians</x:v>
       </x:c>
       <x:c r="I14" s="147" t="n">
-        <x:v>0.08</x:v>
+        <x:v>0.0741</x:v>
       </x:c>
       <x:c r="J14" s="63" t="n">
         <x:v>2033</x:v>
@@ -5882,7 +5882,7 @@
         <x:v>Hospital delivery delay pressure</x:v>
       </x:c>
       <x:c r="L14" s="147" t="n">
-        <x:v>0.02</x:v>
+        <x:v>0.0196</x:v>
       </x:c>
       <x:c r="M14" s="63" t="n">
         <x:v>2034</x:v>
@@ -5914,7 +5914,7 @@
         <x:v>Building electricians</x:v>
       </x:c>
       <x:c r="I15" s="147" t="n">
-        <x:v>3.41</x:v>
+        <x:v>0.7732</x:v>
       </x:c>
       <x:c r="J15" s="63" t="n">
         <x:v>2035</x:v>
@@ -5923,7 +5923,7 @@
         <x:v>Hospital delivery delay pressure</x:v>
       </x:c>
       <x:c r="L15" s="147" t="n">
-        <x:v>8.06</x:v>
+        <x:v>0.8848</x:v>
       </x:c>
       <x:c r="M15" s="63" t="n">
         <x:v>2038</x:v>
@@ -7068,7 +7068,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2976f94d209d4941"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd65803a5e29d4586"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8361,7 +8361,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd9d40f544c834d4c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdfef1e1fbbce4613"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9846,7 +9846,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbf0bdee98204479a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6a4c157bc7064297"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Configure AIIO Sites publication
</commit_message>
<xml_diff>
--- a/public/downloads/AIIO_Alberta_Pilot_0.2.0-dev.xlsx
+++ b/public/downloads/AIIO_Alberta_Pilot_0.2.0-dev.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="1" r:id="Rbdb659b915764819"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="R2e69be1753184ee9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="3" r:id="R48d9bf2bb64540ce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenario Timeline" sheetId="4" r:id="R878b963625d4435b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pressure Results" sheetId="5" r:id="Raad432c252a24166"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="6" r:id="R82df74d975344d32"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Power Overlay" sheetId="7" r:id="Rc5cf58c9d7284230"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI Projects" sheetId="8" r:id="Rda3802c712c44f98"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BCPI Data" sheetId="9" r:id="R15f4ea50a4544859"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="10" r:id="R3aaf5d4183144220"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Checks" sheetId="11" r:id="Rd3445bf53d9a4991"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="1" r:id="R19ceae3698284657"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="R38265614085a4347"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="3" r:id="R73fec3d32db340d9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenario Timeline" sheetId="4" r:id="Rf55f4751bbfe4ca8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pressure Results" sheetId="5" r:id="R29ef336a42e54902"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="6" r:id="R94a6612d8872483f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Power Overlay" sheetId="7" r:id="Raf1a2465c3c7478f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI Projects" sheetId="8" r:id="Racbe8b91b49743ec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BCPI Data" sheetId="9" r:id="R74f42b6c96dc4a4d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="10" r:id="R81c26f731a8a4d52"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Checks" sheetId="11" r:id="R9a5608e937ad4254"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -20,9 +20,9 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:comments xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:authors>
-    <x:author>tc={885C3C5E-B985-4690-9C8E-99BA6A8408ED}</x:author>
-    <x:author>tc={D0D9660F-855D-4070-8175-EF5C94D0680C}</x:author>
-    <x:author>tc={BDA8B6C9-D04B-47AC-864D-F116A333B949}</x:author>
+    <x:author>tc={183655C4-7A6A-449B-8B5F-B7241801F0CE}</x:author>
+    <x:author>tc={CC803864-7B2F-40F0-AC18-832199B9B47A}</x:author>
+    <x:author>tc={1C363C0B-9B56-4323-A318-D92CA8E859B2}</x:author>
   </x:authors>
   <x:commentList>
     <x:comment ref="B5" authorId="0">
@@ -1360,7 +1360,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R59d3b6fddc964358"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rdd94352380a04b8d"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1390,7 +1390,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R9706369f0cd44566"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R53dd8f985a864154"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1418,7 +1418,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:personList xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:person displayName="User" id="{598A9BB0-9441-48FB-A7E6-D669CE17B875}"/>
+  <xltc:person displayName="User" id="{FE60CD91-F20C-47F8-A482-5C073CDA418B}"/>
 </xltc:personList>
 </file>
 
@@ -1691,13 +1691,13 @@
 
 <file path=xl/threadedcomments/threadedcomment.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:ThreadedComments xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:threadedComment ref="B5" dT="2026-08-31T15:29:59.987" personId="{598A9BB0-9441-48FB-A7E6-D669CE17B875}" id="{885C3C5E-B985-4690-9C8E-99BA6A8408ED}">
+  <xltc:threadedComment ref="B5" dT="2026-08-31T15:39:39.317" personId="{FE60CD91-F20C-47F8-A482-5C073CDA418B}" id="{183655C4-7A6A-449B-8B5F-B7241801F0CE}">
     <xltc:text>Scenario-only input. This is not a forecast or a total of committed projects.</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="B10" dT="2026-08-31T15:29:59.988" personId="{598A9BB0-9441-48FB-A7E6-D669CE17B875}" id="{D0D9660F-855D-4070-8175-EF5C94D0680C}">
+  <xltc:threadedComment ref="B10" dT="2026-08-31T15:39:39.319" personId="{FE60CD91-F20C-47F8-A482-5C073CDA418B}" id="{CC803864-7B2F-40F0-AC18-832199B9B47A}">
     <xltc:text>Assumed share of locally captured construction and service demand. Test through sensitivity analysis before interpretation.</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="C24" dT="2026-08-31T15:29:59.988" personId="{598A9BB0-9441-48FB-A7E6-D669CE17B875}" id="{BDA8B6C9-D04B-47AC-864D-F116A333B949}">
+  <xltc:threadedComment ref="C24" dT="2026-08-31T15:39:39.319" personId="{FE60CD91-F20C-47F8-A482-5C073CDA418B}" id="{1C363C0B-9B56-4323-A318-D92CA8E859B2}">
     <xltc:text>IT load is an independent power-case assumption. It is not derived from capital expenditure.</xltc:text>
   </xltc:threadedComment>
 </xltc:ThreadedComments>
@@ -2540,7 +2540,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc2bd8cb1597e4c71"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd77549dc17a04e72"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2648,7 +2648,7 @@
         <x:v>Code commit</x:v>
       </x:c>
       <x:c r="B11" s="160" t="str">
-        <x:v>9812157428b38e578291a31e1a4eb43b6e9d8ec7</x:v>
+        <x:v>5640850cd12d97a5c175e8bb097968a00d93a1ba</x:v>
       </x:c>
       <x:c r="C11" s="63"/>
       <x:c r="D11" s="63"/>
@@ -3592,7 +3592,7 @@
     <x:mergeCell ref="A44:L44"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf55b22b0dcb0489d"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2f91046071dc4d5e"/>
 </x:worksheet>
 </file>
 
@@ -4329,7 +4329,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf0b9b4e894ad4702"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2487ba3b7f94484b"/>
 </x:worksheet>
 </file>
 
@@ -7068,7 +7068,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd65803a5e29d4586"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R90a3f4126e894329"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8361,7 +8361,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdfef1e1fbbce4613"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2d295130f25f4fc5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9846,7 +9846,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6a4c157bc7064297"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rede30f725db54cd7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add Vercel deployment target
</commit_message>
<xml_diff>
--- a/public/downloads/AIIO_Alberta_Pilot_0.2.0-dev.xlsx
+++ b/public/downloads/AIIO_Alberta_Pilot_0.2.0-dev.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="1" r:id="R19ceae3698284657"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="R38265614085a4347"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="3" r:id="R73fec3d32db340d9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenario Timeline" sheetId="4" r:id="Rf55f4751bbfe4ca8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pressure Results" sheetId="5" r:id="R29ef336a42e54902"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="6" r:id="R94a6612d8872483f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Power Overlay" sheetId="7" r:id="Raf1a2465c3c7478f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI Projects" sheetId="8" r:id="Racbe8b91b49743ec"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BCPI Data" sheetId="9" r:id="R74f42b6c96dc4a4d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="10" r:id="R81c26f731a8a4d52"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Checks" sheetId="11" r:id="R9a5608e937ad4254"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="1" r:id="Rb14d36a3af824bee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="R88e2173c23234e43"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="3" r:id="R1b084c00a7b74f03"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenario Timeline" sheetId="4" r:id="R989f600e9007460a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pressure Results" sheetId="5" r:id="Rbbd9dea4cb754227"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="6" r:id="R5e8bfef0b79943bc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Power Overlay" sheetId="7" r:id="R38cbd22646274f49"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI Projects" sheetId="8" r:id="Rc332b03f6ec641e6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BCPI Data" sheetId="9" r:id="R8b84e0d867a64eb9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="10" r:id="R74d558dda3494c4f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Checks" sheetId="11" r:id="R9733fbfc7ad54315"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -20,9 +20,9 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:comments xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:authors>
-    <x:author>tc={183655C4-7A6A-449B-8B5F-B7241801F0CE}</x:author>
-    <x:author>tc={CC803864-7B2F-40F0-AC18-832199B9B47A}</x:author>
-    <x:author>tc={1C363C0B-9B56-4323-A318-D92CA8E859B2}</x:author>
+    <x:author>tc={A7C7E363-0B81-45B8-815B-C92126EF032C}</x:author>
+    <x:author>tc={BC16354B-EB01-443B-8023-EA3E7C0699EE}</x:author>
+    <x:author>tc={6ED81DF5-7C97-45B7-93B7-E23B0E2F26DD}</x:author>
   </x:authors>
   <x:commentList>
     <x:comment ref="B5" authorId="0">
@@ -1360,7 +1360,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rdd94352380a04b8d"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rac607b84629f4bd6"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1390,7 +1390,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R53dd8f985a864154"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R42d2144329a3455e"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1418,7 +1418,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:personList xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:person displayName="User" id="{FE60CD91-F20C-47F8-A482-5C073CDA418B}"/>
+  <xltc:person displayName="User" id="{17BA6477-307F-4590-94E1-F72866056672}"/>
 </xltc:personList>
 </file>
 
@@ -1691,13 +1691,13 @@
 
 <file path=xl/threadedcomments/threadedcomment.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:ThreadedComments xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:threadedComment ref="B5" dT="2026-08-31T15:39:39.317" personId="{FE60CD91-F20C-47F8-A482-5C073CDA418B}" id="{183655C4-7A6A-449B-8B5F-B7241801F0CE}">
+  <xltc:threadedComment ref="B5" dT="2026-08-31T15:43:18.502" personId="{17BA6477-307F-4590-94E1-F72866056672}" id="{A7C7E363-0B81-45B8-815B-C92126EF032C}">
     <xltc:text>Scenario-only input. This is not a forecast or a total of committed projects.</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="B10" dT="2026-08-31T15:39:39.319" personId="{FE60CD91-F20C-47F8-A482-5C073CDA418B}" id="{CC803864-7B2F-40F0-AC18-832199B9B47A}">
+  <xltc:threadedComment ref="B10" dT="2026-08-31T15:43:18.502" personId="{17BA6477-307F-4590-94E1-F72866056672}" id="{BC16354B-EB01-443B-8023-EA3E7C0699EE}">
     <xltc:text>Assumed share of locally captured construction and service demand. Test through sensitivity analysis before interpretation.</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="C24" dT="2026-08-31T15:39:39.319" personId="{FE60CD91-F20C-47F8-A482-5C073CDA418B}" id="{1C363C0B-9B56-4323-A318-D92CA8E859B2}">
+  <xltc:threadedComment ref="C24" dT="2026-08-31T15:43:18.502" personId="{17BA6477-307F-4590-94E1-F72866056672}" id="{6ED81DF5-7C97-45B7-93B7-E23B0E2F26DD}">
     <xltc:text>IT load is an independent power-case assumption. It is not derived from capital expenditure.</xltc:text>
   </xltc:threadedComment>
 </xltc:ThreadedComments>
@@ -2540,7 +2540,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd77549dc17a04e72"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R34cf43e6fe5c4733"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2648,7 +2648,7 @@
         <x:v>Code commit</x:v>
       </x:c>
       <x:c r="B11" s="160" t="str">
-        <x:v>5640850cd12d97a5c175e8bb097968a00d93a1ba</x:v>
+        <x:v>a7a0f7d916a52b9d524072c01b9703d09b1c61b4</x:v>
       </x:c>
       <x:c r="C11" s="63"/>
       <x:c r="D11" s="63"/>
@@ -3592,7 +3592,7 @@
     <x:mergeCell ref="A44:L44"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2f91046071dc4d5e"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf21d203b5f6e4422"/>
 </x:worksheet>
 </file>
 
@@ -4329,7 +4329,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2487ba3b7f94484b"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc088f19610904b7d"/>
 </x:worksheet>
 </file>
 
@@ -7068,7 +7068,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R90a3f4126e894329"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdccd43cb3b8b4a0d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8361,7 +8361,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2d295130f25f4fc5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R21adbae079cd4e46"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9846,7 +9846,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rede30f725db54cd7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2ffdcfedf69a4bde"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Publish AIIO Vercel release bundle
</commit_message>
<xml_diff>
--- a/public/downloads/AIIO_Alberta_Pilot_0.2.0-dev.xlsx
+++ b/public/downloads/AIIO_Alberta_Pilot_0.2.0-dev.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="1" r:id="Rb14d36a3af824bee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="R88e2173c23234e43"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="3" r:id="R1b084c00a7b74f03"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenario Timeline" sheetId="4" r:id="R989f600e9007460a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pressure Results" sheetId="5" r:id="Rbbd9dea4cb754227"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="6" r:id="R5e8bfef0b79943bc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Power Overlay" sheetId="7" r:id="R38cbd22646274f49"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI Projects" sheetId="8" r:id="Rc332b03f6ec641e6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BCPI Data" sheetId="9" r:id="R8b84e0d867a64eb9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="10" r:id="R74d558dda3494c4f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Checks" sheetId="11" r:id="R9733fbfc7ad54315"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="1" r:id="Rc98996d54bd843fa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="Rc029aabe9d1d4c67"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="3" r:id="R204029e4a392460c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenario Timeline" sheetId="4" r:id="R8e5caf987f294562"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pressure Results" sheetId="5" r:id="R85b632f6f7c24bc6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="6" r:id="R1f717ef66ae24f3c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Power Overlay" sheetId="7" r:id="Rbb2af89b25c4478c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI Projects" sheetId="8" r:id="Rca54eb7dea494db3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BCPI Data" sheetId="9" r:id="R1f459be8859f4822"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="10" r:id="R9b2d4aa8c9f34d66"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Checks" sheetId="11" r:id="Re025a22b3bcc4dd3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -20,9 +20,9 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:comments xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:authors>
-    <x:author>tc={A7C7E363-0B81-45B8-815B-C92126EF032C}</x:author>
-    <x:author>tc={BC16354B-EB01-443B-8023-EA3E7C0699EE}</x:author>
-    <x:author>tc={6ED81DF5-7C97-45B7-93B7-E23B0E2F26DD}</x:author>
+    <x:author>tc={02186683-A873-47C9-8199-11BC3CABA619}</x:author>
+    <x:author>tc={8C500287-9B1E-4422-9C55-D7D7D5FC7B9A}</x:author>
+    <x:author>tc={461F2A1B-9EE1-4F75-BA51-84A5F45683CB}</x:author>
   </x:authors>
   <x:commentList>
     <x:comment ref="B5" authorId="0">
@@ -1360,7 +1360,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rac607b84629f4bd6"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re5d7d6735e584c21"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1390,7 +1390,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R42d2144329a3455e"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R45223fa0e5ff4182"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1418,7 +1418,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:personList xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:person displayName="User" id="{17BA6477-307F-4590-94E1-F72866056672}"/>
+  <xltc:person displayName="User" id="{643F83D7-4D12-47F4-9AD7-59DD62B077D0}"/>
 </xltc:personList>
 </file>
 
@@ -1691,13 +1691,13 @@
 
 <file path=xl/threadedcomments/threadedcomment.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:ThreadedComments xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:threadedComment ref="B5" dT="2026-08-31T15:43:18.502" personId="{17BA6477-307F-4590-94E1-F72866056672}" id="{A7C7E363-0B81-45B8-815B-C92126EF032C}">
+  <xltc:threadedComment ref="B5" dT="2026-08-31T17:20:31.976" personId="{643F83D7-4D12-47F4-9AD7-59DD62B077D0}" id="{02186683-A873-47C9-8199-11BC3CABA619}">
     <xltc:text>Scenario-only input. This is not a forecast or a total of committed projects.</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="B10" dT="2026-08-31T15:43:18.502" personId="{17BA6477-307F-4590-94E1-F72866056672}" id="{BC16354B-EB01-443B-8023-EA3E7C0699EE}">
+  <xltc:threadedComment ref="B10" dT="2026-08-31T17:20:31.978" personId="{643F83D7-4D12-47F4-9AD7-59DD62B077D0}" id="{8C500287-9B1E-4422-9C55-D7D7D5FC7B9A}">
     <xltc:text>Assumed share of locally captured construction and service demand. Test through sensitivity analysis before interpretation.</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="C24" dT="2026-08-31T15:43:18.502" personId="{17BA6477-307F-4590-94E1-F72866056672}" id="{6ED81DF5-7C97-45B7-93B7-E23B0E2F26DD}">
+  <xltc:threadedComment ref="C24" dT="2026-08-31T17:20:31.978" personId="{643F83D7-4D12-47F4-9AD7-59DD62B077D0}" id="{461F2A1B-9EE1-4F75-BA51-84A5F45683CB}">
     <xltc:text>IT load is an independent power-case assumption. It is not derived from capital expenditure.</xltc:text>
   </xltc:threadedComment>
 </xltc:ThreadedComments>
@@ -2540,7 +2540,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R34cf43e6fe5c4733"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R48088b4accc04ce0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2648,7 +2648,7 @@
         <x:v>Code commit</x:v>
       </x:c>
       <x:c r="B11" s="160" t="str">
-        <x:v>a7a0f7d916a52b9d524072c01b9703d09b1c61b4</x:v>
+        <x:v>a2a1d25c011d71e489565b29ab48327a688b9b2e</x:v>
       </x:c>
       <x:c r="C11" s="63"/>
       <x:c r="D11" s="63"/>
@@ -3592,7 +3592,7 @@
     <x:mergeCell ref="A44:L44"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf21d203b5f6e4422"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R910ff13d6b5642a0"/>
 </x:worksheet>
 </file>
 
@@ -4329,7 +4329,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc088f19610904b7d"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R82ef0979042e4847"/>
 </x:worksheet>
 </file>
 
@@ -7068,7 +7068,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rdccd43cb3b8b4a0d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0da134b954a241db"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8361,7 +8361,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R21adbae079cd4e46"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8e93296a2cc54d0d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9846,7 +9846,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2ffdcfedf69a4bde"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb79415ff29334f0e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Publish CI-verified AIIO release bundle
</commit_message>
<xml_diff>
--- a/public/downloads/AIIO_Alberta_Pilot_0.2.0-dev.xlsx
+++ b/public/downloads/AIIO_Alberta_Pilot_0.2.0-dev.xlsx
@@ -2,17 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="1" r:id="Rc98996d54bd843fa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="Rc029aabe9d1d4c67"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="3" r:id="R204029e4a392460c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenario Timeline" sheetId="4" r:id="R8e5caf987f294562"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pressure Results" sheetId="5" r:id="R85b632f6f7c24bc6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="6" r:id="R1f717ef66ae24f3c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Power Overlay" sheetId="7" r:id="Rbb2af89b25c4478c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI Projects" sheetId="8" r:id="Rca54eb7dea494db3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BCPI Data" sheetId="9" r:id="R1f459be8859f4822"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="10" r:id="R9b2d4aa8c9f34d66"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Checks" sheetId="11" r:id="Re025a22b3bcc4dd3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="1" r:id="Rbebc61b258874d53"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="Rfe83556de4f24429"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assumptions" sheetId="3" r:id="R49553869b0524143"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenario Timeline" sheetId="4" r:id="Radfa2848a7c142be"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pressure Results" sheetId="5" r:id="Rfcff4f0939dc496a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="6" r:id="R7df9161992994064"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Power Overlay" sheetId="7" r:id="R005b3f03197a416c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI Projects" sheetId="8" r:id="Rff70d5de66784250"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BCPI Data" sheetId="9" r:id="Rfbae9cc766ec4123"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="10" r:id="Rb2be2287e1df40e3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Release Checks" sheetId="11" r:id="Ree1c0d3cd53c472c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -20,9 +20,9 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:comments xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:authors>
-    <x:author>tc={02186683-A873-47C9-8199-11BC3CABA619}</x:author>
-    <x:author>tc={8C500287-9B1E-4422-9C55-D7D7D5FC7B9A}</x:author>
-    <x:author>tc={461F2A1B-9EE1-4F75-BA51-84A5F45683CB}</x:author>
+    <x:author>tc={BE73263F-C5ED-48B9-A05E-1FF05F666122}</x:author>
+    <x:author>tc={9E65F65F-8F1E-42C8-A2CD-2FAAB011C9C7}</x:author>
+    <x:author>tc={C8110CD7-4295-4AE0-B911-DC093BAD94B2}</x:author>
   </x:authors>
   <x:commentList>
     <x:comment ref="B5" authorId="0">
@@ -1360,7 +1360,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re5d7d6735e584c21"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R867a9e34c86b46b5"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1390,7 +1390,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R45223fa0e5ff4182"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R115e257585184529"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1418,7 +1418,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:personList xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:person displayName="User" id="{643F83D7-4D12-47F4-9AD7-59DD62B077D0}"/>
+  <xltc:person displayName="User" id="{C84F0700-C9E3-4F48-8770-F22C6C61C332}"/>
 </xltc:personList>
 </file>
 
@@ -1691,13 +1691,13 @@
 
 <file path=xl/threadedcomments/threadedcomment.xml><?xml version="1.0" encoding="utf-8"?>
 <xltc:ThreadedComments xmlns:xltc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <xltc:threadedComment ref="B5" dT="2026-08-31T17:20:31.976" personId="{643F83D7-4D12-47F4-9AD7-59DD62B077D0}" id="{02186683-A873-47C9-8199-11BC3CABA619}">
+  <xltc:threadedComment ref="B5" dT="2026-08-31T17:46:03.256" personId="{C84F0700-C9E3-4F48-8770-F22C6C61C332}" id="{BE73263F-C5ED-48B9-A05E-1FF05F666122}">
     <xltc:text>Scenario-only input. This is not a forecast or a total of committed projects.</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="B10" dT="2026-08-31T17:20:31.978" personId="{643F83D7-4D12-47F4-9AD7-59DD62B077D0}" id="{8C500287-9B1E-4422-9C55-D7D7D5FC7B9A}">
+  <xltc:threadedComment ref="B10" dT="2026-08-31T17:46:03.257" personId="{C84F0700-C9E3-4F48-8770-F22C6C61C332}" id="{9E65F65F-8F1E-42C8-A2CD-2FAAB011C9C7}">
     <xltc:text>Assumed share of locally captured construction and service demand. Test through sensitivity analysis before interpretation.</xltc:text>
   </xltc:threadedComment>
-  <xltc:threadedComment ref="C24" dT="2026-08-31T17:20:31.978" personId="{643F83D7-4D12-47F4-9AD7-59DD62B077D0}" id="{461F2A1B-9EE1-4F75-BA51-84A5F45683CB}">
+  <xltc:threadedComment ref="C24" dT="2026-08-31T17:46:03.257" personId="{C84F0700-C9E3-4F48-8770-F22C6C61C332}" id="{C8110CD7-4295-4AE0-B911-DC093BAD94B2}">
     <xltc:text>IT load is an independent power-case assumption. It is not derived from capital expenditure.</xltc:text>
   </xltc:threadedComment>
 </xltc:ThreadedComments>
@@ -2540,7 +2540,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R48088b4accc04ce0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R910585979a0440a9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2648,7 +2648,7 @@
         <x:v>Code commit</x:v>
       </x:c>
       <x:c r="B11" s="160" t="str">
-        <x:v>a2a1d25c011d71e489565b29ab48327a688b9b2e</x:v>
+        <x:v>485902bd50faea5e0dc62227d7302762d481a44e</x:v>
       </x:c>
       <x:c r="C11" s="63"/>
       <x:c r="D11" s="63"/>
@@ -3592,7 +3592,7 @@
     <x:mergeCell ref="A44:L44"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R910ff13d6b5642a0"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R056a9f4a08534db8"/>
 </x:worksheet>
 </file>
 
@@ -4329,7 +4329,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R82ef0979042e4847"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra31deeb3ddcb4715"/>
 </x:worksheet>
 </file>
 
@@ -7068,7 +7068,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0da134b954a241db"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R65ffe6a354d34ca0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8361,7 +8361,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8e93296a2cc54d0d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2242bd843c014a5f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9846,7 +9846,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb79415ff29334f0e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3e0bc8040375407e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>